<commit_message>
updated data to 5/9/2025; used Adj CLOSE for price.
</commit_message>
<xml_diff>
--- a/template_etf_output.xlsx
+++ b/template_etf_output.xlsx
@@ -489,7 +489,7 @@
         <v>0.0355</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0609</v>
+        <v>0.0606</v>
       </c>
     </row>
     <row r="3">
@@ -515,7 +515,7 @@
         <v>0.0336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0604</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="4">
@@ -541,7 +541,7 @@
         <v>0.0636</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1694</v>
+        <v>0.169</v>
       </c>
     </row>
     <row r="5">
@@ -567,7 +567,7 @@
         <v>0.08</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1981</v>
+        <v>0.1972</v>
       </c>
     </row>
     <row r="6">
@@ -593,7 +593,7 @@
         <v>0.08309999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0746</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="7">
@@ -619,7 +619,7 @@
         <v>0.1963</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1899</v>
+        <v>0.1896</v>
       </c>
     </row>
     <row r="8">
@@ -645,7 +645,7 @@
         <v>0.0434</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0586</v>
+        <v>0.0583</v>
       </c>
     </row>
     <row r="9">
@@ -671,7 +671,7 @@
         <v>0.1348</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2128</v>
+        <v>0.2121</v>
       </c>
     </row>
     <row r="10">
@@ -697,7 +697,7 @@
         <v>0.1215</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2003</v>
+        <v>0.1979</v>
       </c>
     </row>
     <row r="11">
@@ -723,7 +723,7 @@
         <v>0.1927</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1915</v>
+        <v>0.1913</v>
       </c>
     </row>
     <row r="12">
@@ -749,7 +749,7 @@
         <v>0.1656</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1548</v>
+        <v>0.1542</v>
       </c>
     </row>
     <row r="13">
@@ -775,7 +775,7 @@
         <v>0.1287</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1804</v>
+        <v>0.1799</v>
       </c>
     </row>
     <row r="14">
@@ -801,7 +801,7 @@
         <v>0.2</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1519</v>
+        <v>0.1583</v>
       </c>
     </row>
   </sheetData>
@@ -878,7 +878,7 @@
         <v>0.0355</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0609</v>
+        <v>0.0606</v>
       </c>
       <c r="G2" t="n">
         <v>0.5831</v>
@@ -907,7 +907,7 @@
         <v>0.0336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0604</v>
+        <v>0.06</v>
       </c>
       <c r="G3" t="n">
         <v>0.5567</v>
@@ -936,7 +936,7 @@
         <v>0.0636</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1694</v>
+        <v>0.169</v>
       </c>
       <c r="G4" t="n">
         <v>0.3753</v>
@@ -965,7 +965,7 @@
         <v>0.08</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1981</v>
+        <v>0.1972</v>
       </c>
       <c r="G5" t="n">
         <v>0.4037</v>
@@ -994,7 +994,7 @@
         <v>0.08309999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0746</v>
+        <v>0.074</v>
       </c>
       <c r="G6" t="n">
         <v>1.1136</v>
@@ -1023,7 +1023,7 @@
         <v>0.1963</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1899</v>
+        <v>0.1896</v>
       </c>
       <c r="G7" t="n">
         <v>1.0338</v>
@@ -1052,7 +1052,7 @@
         <v>0.0434</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0586</v>
+        <v>0.0583</v>
       </c>
       <c r="G8" t="n">
         <v>0.7401</v>
@@ -1081,7 +1081,7 @@
         <v>0.1348</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2128</v>
+        <v>0.2121</v>
       </c>
       <c r="G9" t="n">
         <v>0.6334</v>
@@ -1110,7 +1110,7 @@
         <v>0.1215</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2003</v>
+        <v>0.1979</v>
       </c>
       <c r="G10" t="n">
         <v>0.6064000000000001</v>
@@ -1139,7 +1139,7 @@
         <v>0.1927</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1915</v>
+        <v>0.1913</v>
       </c>
       <c r="G11" t="n">
         <v>1.0062</v>
@@ -1168,7 +1168,7 @@
         <v>0.1656</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1548</v>
+        <v>0.1542</v>
       </c>
       <c r="G12" t="n">
         <v>1.07</v>
@@ -1197,7 +1197,7 @@
         <v>0.1287</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1804</v>
+        <v>0.1799</v>
       </c>
       <c r="G13" t="n">
         <v>0.7134</v>
@@ -1226,7 +1226,7 @@
         <v>0.2</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1519</v>
+        <v>0.1583</v>
       </c>
       <c r="G14" t="n">
         <v>1.3163</v>
@@ -1301,7 +1301,7 @@
         <v>0.0355</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0609</v>
+        <v>0.0606</v>
       </c>
     </row>
     <row r="3">
@@ -1327,7 +1327,7 @@
         <v>0.0336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0604</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="4">
@@ -1353,7 +1353,7 @@
         <v>0.0636</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1694</v>
+        <v>0.169</v>
       </c>
     </row>
     <row r="5">
@@ -1379,7 +1379,7 @@
         <v>0.08</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1981</v>
+        <v>0.1972</v>
       </c>
     </row>
     <row r="6">
@@ -1405,7 +1405,7 @@
         <v>0.08309999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0746</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="7">
@@ -1431,7 +1431,7 @@
         <v>0.1963</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1899</v>
+        <v>0.1896</v>
       </c>
     </row>
     <row r="8">
@@ -1457,7 +1457,7 @@
         <v>0.0434</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0586</v>
+        <v>0.0583</v>
       </c>
     </row>
     <row r="9">
@@ -1483,7 +1483,7 @@
         <v>0.1348</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2128</v>
+        <v>0.2121</v>
       </c>
     </row>
     <row r="10">
@@ -1509,7 +1509,7 @@
         <v>0.1215</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2003</v>
+        <v>0.1979</v>
       </c>
     </row>
     <row r="11">
@@ -1535,7 +1535,7 @@
         <v>0.1927</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1915</v>
+        <v>0.1913</v>
       </c>
     </row>
     <row r="12">
@@ -1561,7 +1561,7 @@
         <v>0.1656</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1548</v>
+        <v>0.1542</v>
       </c>
     </row>
     <row r="13">
@@ -1587,7 +1587,7 @@
         <v>0.1287</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1804</v>
+        <v>0.1799</v>
       </c>
     </row>
     <row r="14">
@@ -1613,7 +1613,7 @@
         <v>0.2</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1519</v>
+        <v>0.1583</v>
       </c>
     </row>
   </sheetData>
@@ -1685,7 +1685,7 @@
         <v>0.0355</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0609</v>
+        <v>0.0606</v>
       </c>
     </row>
     <row r="3">
@@ -1711,7 +1711,7 @@
         <v>0.0336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0604</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="4">
@@ -1737,7 +1737,7 @@
         <v>0.0636</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1694</v>
+        <v>0.169</v>
       </c>
     </row>
     <row r="5">
@@ -1763,7 +1763,7 @@
         <v>0.08</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1981</v>
+        <v>0.1972</v>
       </c>
     </row>
     <row r="6">
@@ -1789,7 +1789,7 @@
         <v>0.08309999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0746</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="7">
@@ -1815,7 +1815,7 @@
         <v>0.1963</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1899</v>
+        <v>0.1896</v>
       </c>
     </row>
     <row r="8">
@@ -1841,7 +1841,7 @@
         <v>0.0434</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0586</v>
+        <v>0.0583</v>
       </c>
     </row>
     <row r="9">
@@ -1867,7 +1867,7 @@
         <v>0.1348</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2128</v>
+        <v>0.2121</v>
       </c>
     </row>
     <row r="10">
@@ -1893,7 +1893,7 @@
         <v>0.1215</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2003</v>
+        <v>0.1979</v>
       </c>
     </row>
     <row r="11">
@@ -1919,7 +1919,7 @@
         <v>0.1927</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1915</v>
+        <v>0.1913</v>
       </c>
     </row>
     <row r="12">
@@ -1945,7 +1945,7 @@
         <v>0.1656</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1548</v>
+        <v>0.1542</v>
       </c>
     </row>
     <row r="13">
@@ -1971,7 +1971,7 @@
         <v>0.1287</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1804</v>
+        <v>0.1799</v>
       </c>
     </row>
     <row r="14">
@@ -1997,7 +1997,7 @@
         <v>0.2</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1519</v>
+        <v>0.1583</v>
       </c>
     </row>
   </sheetData>
@@ -2074,7 +2074,7 @@
         <v>0.0355</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0609</v>
+        <v>0.0606</v>
       </c>
       <c r="G2" t="n">
         <v>0.0025</v>
@@ -2103,7 +2103,7 @@
         <v>0.0336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0604</v>
+        <v>0.06</v>
       </c>
       <c r="G3" t="n">
         <v>0.0026</v>
@@ -2132,7 +2132,7 @@
         <v>0.0636</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1694</v>
+        <v>0.169</v>
       </c>
       <c r="G4" t="n">
         <v>0.0027</v>
@@ -2161,7 +2161,7 @@
         <v>0.08</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1981</v>
+        <v>0.1972</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -2190,7 +2190,7 @@
         <v>0.08309999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0746</v>
+        <v>0.074</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -2219,7 +2219,7 @@
         <v>0.1963</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1899</v>
+        <v>0.1896</v>
       </c>
       <c r="G7" t="n">
         <v>0.0125</v>
@@ -2248,7 +2248,7 @@
         <v>0.0434</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0586</v>
+        <v>0.0583</v>
       </c>
       <c r="G8" t="n">
         <v>0.0021</v>
@@ -2277,7 +2277,7 @@
         <v>0.1348</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2128</v>
+        <v>0.2121</v>
       </c>
       <c r="G9" t="n">
         <v>0.0102</v>
@@ -2306,7 +2306,7 @@
         <v>0.1215</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2003</v>
+        <v>0.1979</v>
       </c>
       <c r="G10" t="n">
         <v>0.0026</v>
@@ -2335,7 +2335,7 @@
         <v>0.1927</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1915</v>
+        <v>0.1913</v>
       </c>
       <c r="G11" t="n">
         <v>0.0115</v>
@@ -2364,7 +2364,7 @@
         <v>0.1656</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1548</v>
+        <v>0.1542</v>
       </c>
       <c r="G12" t="n">
         <v>0.0201</v>
@@ -2393,7 +2393,7 @@
         <v>0.1287</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1804</v>
+        <v>0.1799</v>
       </c>
       <c r="G13" t="n">
         <v>0.0225</v>
@@ -2422,7 +2422,7 @@
         <v>0.2</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1519</v>
+        <v>0.1583</v>
       </c>
       <c r="G14" t="n">
         <v>0.0118</v>
@@ -2502,7 +2502,7 @@
         <v>0.0355</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0609</v>
+        <v>0.0606</v>
       </c>
       <c r="G2" t="n">
         <v>0.0205</v>
@@ -2531,7 +2531,7 @@
         <v>0.0336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0604</v>
+        <v>0.06</v>
       </c>
       <c r="G3" t="n">
         <v>0.0203</v>
@@ -2560,7 +2560,7 @@
         <v>0.0636</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1694</v>
+        <v>0.169</v>
       </c>
       <c r="G4" t="n">
         <v>0.0622</v>
@@ -2589,7 +2589,7 @@
         <v>0.08</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1981</v>
+        <v>0.1972</v>
       </c>
       <c r="G5" t="n">
         <v>0.0699</v>
@@ -2618,7 +2618,7 @@
         <v>0.08309999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0746</v>
+        <v>0.074</v>
       </c>
       <c r="G6" t="n">
         <v>0.024</v>
@@ -2647,7 +2647,7 @@
         <v>0.1963</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1899</v>
+        <v>0.1896</v>
       </c>
       <c r="G7" t="n">
         <v>0.0615</v>
@@ -2676,7 +2676,7 @@
         <v>0.0434</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0586</v>
+        <v>0.0583</v>
       </c>
       <c r="G8" t="n">
         <v>0.0194</v>
@@ -2705,7 +2705,7 @@
         <v>0.1348</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2128</v>
+        <v>0.2121</v>
       </c>
       <c r="G9" t="n">
         <v>0.0721</v>
@@ -2734,7 +2734,7 @@
         <v>0.1215</v>
       </c>
       <c r="F10" t="n">
-        <v>0.2003</v>
+        <v>0.1979</v>
       </c>
       <c r="G10" t="n">
         <v>0.0672</v>
@@ -2763,7 +2763,7 @@
         <v>0.1927</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1915</v>
+        <v>0.1913</v>
       </c>
       <c r="G11" t="n">
         <v>0.0619</v>
@@ -2792,7 +2792,7 @@
         <v>0.1656</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1548</v>
+        <v>0.1542</v>
       </c>
       <c r="G12" t="n">
         <v>0.0513</v>
@@ -2821,7 +2821,7 @@
         <v>0.1287</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1804</v>
+        <v>0.1799</v>
       </c>
       <c r="G13" t="n">
         <v>0.0599</v>
@@ -2850,7 +2850,7 @@
         <v>0.2</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1519</v>
+        <v>0.1583</v>
       </c>
       <c r="G14" t="n">
         <v>0.0478</v>

</xml_diff>